<commit_message>
01-10 after bug fixes
</commit_message>
<xml_diff>
--- a/flipkart_automation/inputs/product.xlsx
+++ b/flipkart_automation/inputs/product.xlsx
@@ -1,124 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\Admin\OneDrive - StayAhead\Documents\Demo_Sruthy\flipkart_automation\inputs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C760DB-7AB1-4EAD-B095-385A21BCC40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89406741-7B21-4071-A0A3-6DE1F1E57DAE}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Product</t>
-  </si>
-  <si>
-    <t>Customer Ratings</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>Found/Not</t>
-  </si>
-  <si>
-    <t>Laptop</t>
-  </si>
-  <si>
-    <t>Headphone</t>
-  </si>
-  <si>
-    <t>Speaker</t>
-  </si>
-  <si>
-    <t>ipad</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>sruthr1810@gmail.com</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>David</t>
-  </si>
-  <si>
-    <t>Xavier</t>
-  </si>
-  <si>
-    <t>Fernandres</t>
-  </si>
-  <si>
-    <t>Tony</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -132,26 +57,87 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -471,126 +457,200 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB6DB1CA-E020-480C-9FEB-078CB80FE82B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
-    <col min="6" max="6" width="21.42578125" customWidth="1"/>
+    <col width="12.7109375" customWidth="1" min="1" max="1"/>
+    <col width="11.42578125" customWidth="1" min="2" max="2"/>
+    <col width="16.28515625" customWidth="1" min="4" max="4"/>
+    <col width="17.5703125" customWidth="1" min="5" max="5"/>
+    <col width="21.42578125" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Customer Ratings</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Found/Not</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>smart watch</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D2" t="n">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>sruthr1810@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>9</v>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>sruthr1810@gmail.com</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>40000</v>
-      </c>
-      <c r="D2">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Xavier</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Headphone</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D4" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>10</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>sruthr1810@gmail.com</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3">
-        <v>20000</v>
-      </c>
-      <c r="D3">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fernandres</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Speaker</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D5" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>10</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>sruthr1810@gmail.com</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4">
-        <v>2000</v>
-      </c>
-      <c r="D4">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tony</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ipad</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D6" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>2000</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>30000</v>
-      </c>
-      <c r="D6">
-        <v>3</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>10</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>sruthr1810@gmail.com</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{92B26883-498D-4837-A132-E10F975938BD}"/>
-    <hyperlink ref="F3:F6" r:id="rId2" display="sruthr1810@gmail.com" xr:uid="{A0EE5FC3-A091-42EC-A176-7CF5FB8973A8}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" display="sruthr1810@gmail.com" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" display="sruthr1810@gmail.com" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" display="sruthr1810@gmail.com" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" display="sruthr1810@gmail.com" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
After adding to cart
</commit_message>
<xml_diff>
--- a/flipkart_automation/inputs/product.xlsx
+++ b/flipkart_automation/inputs/product.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2055" yWindow="1905" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -33,7 +33,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,7 +42,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF0000"/>
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,9 +66,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" min="1" max="1"/>
@@ -470,6 +475,8 @@
     <col width="16.28515625" customWidth="1" min="4" max="4"/>
     <col width="17.5703125" customWidth="1" min="5" max="5"/>
     <col width="21.42578125" customWidth="1" min="6" max="6"/>
+    <col width="40.28515625" customWidth="1" min="7" max="7"/>
+    <col width="23.42578125" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,162 +502,202 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Found/Not</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
           <t>Email</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>John</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>smart watch</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="1" t="n">
         <v>5000</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Found</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="1" t="n">
         <v>20000</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>sruthyr1810@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>sruthr1810@gmail.com</t>
-        </is>
-      </c>
+      <c r="H3" s="1" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Xavier</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Headphone</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Found</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Fernandres</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Speaker</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="1" t="n">
         <v>3000</v>
       </c>
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Found</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="D5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Tony</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ipad</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>30000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Found</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Shirt</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>40/S</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" display="sruthr1810@gmail.com" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" display="sruthr1810@gmail.com" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" display="sruthr1810@gmail.com" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" display="sruthr1810@gmail.com" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
After fixing the size
</commit_message>
<xml_diff>
--- a/flipkart_automation/inputs/product.xlsx
+++ b/flipkart_automation/inputs/product.xlsx
@@ -33,7 +33,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -42,7 +42,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -64,11 +74,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -522,174 +537,194 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>John</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>smart watch</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="5" t="n">
         <v>5000</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="n"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>1 of 1 products added to cart</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="5" t="n">
         <v>20000</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>sruthyr1810@gmail.com</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>1 of 1 products added to cart</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Xavier</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Headphone</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>1 of 1 products added to cart</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Fernandres</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Speaker</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="C5" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="H5" s="1" t="n"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Products found but none could be added to cart | TRIGGR Horizon 16 with Dual Drivers, 7Hrs Playtime, MEMS Mic, TWS Function 16 W Bluetooth Speaker: Add to cart button not found (neither text nor icon)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Tony</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Shirt</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>40/S</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>S,40</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>sruthr1810@gmail.com</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>1 of 1 products added to cart</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>